<commit_message>
Lambda 2023-04-06 修改excel 模板
</commit_message>
<xml_diff>
--- a/erp-server/erp-server-scm/src/main/resources/excel/purchasePriceDetail.xlsx
+++ b/erp-server/erp-server-scm/src/main/resources/excel/purchasePriceDetail.xlsx
@@ -16,11 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="8">
-  <si>
-    <t>仓库名称</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7" uniqueCount="7">
   <si>
     <t>采购交期(天)</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -415,24 +411,23 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:H1"/>
+  <dimension ref="A1:G1"/>
   <sheetFormatPr defaultRowHeight="13.5" x14ac:dyDescent="0.15"/>
   <cols>
-    <col min="1" max="1" width="27.875" customWidth="1"/>
-    <col min="2" max="2" width="37" customWidth="1"/>
-    <col min="3" max="3" width="22.875" customWidth="1"/>
-    <col min="4" max="5" width="17.625" customWidth="1"/>
-    <col min="6" max="6" width="30.125" customWidth="1"/>
-    <col min="7" max="7" width="25.75" customWidth="1"/>
-    <col min="8" max="8" width="19.5" customWidth="1"/>
+    <col min="1" max="1" width="37" customWidth="1"/>
+    <col min="2" max="2" width="22.875" customWidth="1"/>
+    <col min="3" max="4" width="17.625" customWidth="1"/>
+    <col min="5" max="5" width="30.125" customWidth="1"/>
+    <col min="6" max="6" width="25.75" customWidth="1"/>
+    <col min="7" max="7" width="19.5" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" s="2" customFormat="1" ht="21.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A1" s="1" t="s">
+    <row r="1" spans="1:7" s="2" customFormat="1" ht="21.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A1" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>0</v>
-      </c>
-      <c r="B1" s="3" t="s">
-        <v>7</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>1</v>
@@ -440,7 +435,7 @@
       <c r="D1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" s="3" t="s">
         <v>3</v>
       </c>
       <c r="F1" s="3" t="s">
@@ -448,9 +443,6 @@
       </c>
       <c r="G1" s="3" t="s">
         <v>5</v>
-      </c>
-      <c r="H1" s="3" t="s">
-        <v>6</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Lambda 2023-04-07  sys 修改问题
</commit_message>
<xml_diff>
--- a/erp-server/erp-server-scm/src/main/resources/excel/purchasePriceDetail.xlsx
+++ b/erp-server/erp-server-scm/src/main/resources/excel/purchasePriceDetail.xlsx
@@ -57,6 +57,10 @@
     </r>
   </si>
   <si>
+    <t>币种</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
     <r>
       <t>*</t>
     </r>
@@ -70,12 +74,30 @@
       </rPr>
       <t>税率(%)</t>
     </r>
-  </si>
-  <si>
-    <t>生效日期</t>
-  </si>
-  <si>
-    <t>币种</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="宋体"/>
+        <family val="3"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>*</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="宋体"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>生效日期</t>
+    </r>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
 </sst>
@@ -83,7 +105,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <fonts count="5">
+  <fonts count="7">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -113,6 +135,22 @@
     </font>
     <font>
       <sz val="9"/>
+      <name val="宋体"/>
+      <family val="3"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
+      <name val="宋体"/>
+      <family val="3"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
       <name val="宋体"/>
       <family val="3"/>
       <charset val="134"/>
@@ -163,10 +201,10 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -497,14 +535,14 @@
       <c r="E1" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="5" t="s">
+      <c r="F1" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="5" t="s">
         <v>7</v>
-      </c>
-      <c r="G1" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="H1" s="4" t="s">
-        <v>6</v>
       </c>
     </row>
   </sheetData>

</xml_diff>